<commit_message>
Switch coverage analysis to Sendungsebene (Auftragsnummer <-> sendungs_nr)
Matching now purely on Sendungsnummer instead of Rechnungsnummer.
Updated columns: BI PRE-Sendungen, PDF Sendungen, PDF Positionen,
Matches, BI ohne PDF (abs/%), PDF ohne BI (abs/%).

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/00_coverage_bi_vs_pdf.xlsx
+++ b/output/billing_report/00_coverage_bi_vs_pdf.xlsx
@@ -41,7 +41,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,11 +56,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -108,18 +103,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -487,23 +470,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -526,60 +506,45 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>BI PRE-Zeilen</t>
+          <t>BI PRE-Sendungen</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BI uni. RechNr</t>
+          <t>PDF Sendungen</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>PDF Rechnungen</t>
+          <t>PDF Positionen</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PDF Positionen</t>
+          <t>Matches</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Matches (RechNr)</t>
+          <t>BI ohne PDF (abs)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Matches (SendNr)</t>
+          <t>BI ohne PDF (%)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>BI-Zeilen mit Match</t>
+          <t>PDF ohne BI (abs)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>BI ohne PDF (abs)</t>
+          <t>PDF ohne BI (%)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>BI ohne PDF (%)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>PDF ohne BI (abs)</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>PDF ohne BI (%)</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Anmerkung</t>
         </is>
@@ -600,38 +565,29 @@
         <v>2104</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>2074</v>
+        <v>4353</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>4214</v>
+        <v>4541</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>4541</v>
+        <v>1598</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1568</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>1598</v>
+        <v>506</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>24</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>1598</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>506</v>
-      </c>
-      <c r="K3" s="5" t="n">
-        <v>24</v>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>2859</v>
-      </c>
-      <c r="M3" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
-        <is>
-          <t>PDF hat 2140 mehr RechNr als BI → PDFs ohne BI-Eintrag</t>
+        <v>2755</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>2249 mehr PDF-Sendungen als BI-Sendungen → PDFs aus anderen Perioden/Kunden</t>
         </is>
       </c>
     </row>
@@ -650,38 +606,29 @@
         <v>1041</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>187</v>
+        <v>1310</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>718</v>
+        <v>1347</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1347</v>
+        <v>201</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>115</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>201</v>
+        <v>840</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>80.7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>586</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>455</v>
-      </c>
-      <c r="K4" s="5" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>1019</v>
-      </c>
-      <c r="M4" s="5" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="N4" s="6" t="inlineStr">
-        <is>
-          <t>BI 6 Zeilen/RechNr, PDF 1.9 Pos/RechNr → PDF ist aggregiert</t>
+        <v>1109</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Ø 1.0 PDF-Positionen/Sendung</t>
         </is>
       </c>
     </row>
@@ -700,38 +647,29 @@
         <v>1839</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>80</v>
+        <v>297</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>152</v>
+        <v>382</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>382</v>
+        <v>157</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>157</v>
+        <v>1682</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>91.5</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1365</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>474</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>167</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>BI 23 Zeilen/RechNr, PDF 2.5 Pos/RechNr → PDF ist aggregiert</t>
+        <v>140</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>1542 mehr BI-Sendungen als PDF-Sendungen → fehlende PDFs</t>
         </is>
       </c>
     </row>
@@ -750,38 +688,29 @@
         <v>717</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>90</v>
+        <v>144</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>144</v>
+        <v>66</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>66</v>
+        <v>651</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>90.8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>97</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>620</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>86.5</v>
-      </c>
-      <c r="L6" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>54.2</v>
       </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>BI hat 71 mehr RechNr als PDF → fehlende PDFs</t>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>573 mehr BI-Sendungen als PDF-Sendungen → fehlende PDFs</t>
         </is>
       </c>
     </row>
@@ -800,88 +729,70 @@
         <v>77</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>73</v>
+        <v>123</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>77</v>
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>77</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>37.4</v>
       </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>PDF hat 45 mehr RechNr als BI → PDFs ohne BI-Eintrag</t>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>46 mehr PDF-Sendungen als BI-Sendungen → PDFs aus anderen Perioden/Kunden</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>HERMA GmbH</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>423650</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="4" t="n">
         <v>4035</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>289</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>275</v>
-      </c>
-      <c r="F8" s="8" t="n">
+      <c r="D8" s="4" t="n">
+        <v>428</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>442</v>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>192</v>
-      </c>
-      <c r="H8" s="8" t="n">
+      <c r="F8" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="I8" s="8" t="n">
-        <v>2899</v>
-      </c>
-      <c r="J8" s="8" t="n">
-        <v>1136</v>
-      </c>
-      <c r="K8" s="9" t="n">
-        <v>28.2</v>
-      </c>
-      <c r="L8" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="M8" s="9" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="N8" s="10" t="inlineStr">
-        <is>
-          <t>BI 14 Zeilen/RechNr, PDF 1.6 Pos/RechNr → PDF ist aggregiert</t>
+      <c r="G8" s="4" t="n">
+        <v>3712</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>3607 mehr BI-Sendungen als PDF-Sendungen → fehlende PDFs</t>
         </is>
       </c>
     </row>
@@ -900,38 +811,29 @@
         <v>1922</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>212</v>
+        <v>4479</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>540</v>
+        <v>4489</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4489</v>
+        <v>1442</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>1442</v>
+        <v>480</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>25</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>1442</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>480</v>
-      </c>
-      <c r="K9" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>2881</v>
-      </c>
-      <c r="M9" s="5" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>PDF hat 328 mehr RechNr als BI → PDFs ohne BI-Eintrag</t>
+        <v>3037</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>2557 mehr PDF-Sendungen als BI-Sendungen → PDFs aus anderen Perioden/Kunden</t>
         </is>
       </c>
     </row>
@@ -950,38 +852,29 @@
         <v>912</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>80</v>
+        <v>4990</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>445</v>
+        <v>5126</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>5126</v>
+        <v>658</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>658</v>
+        <v>254</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>27.9</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>658</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>254</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>4380</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>85.40000000000001</v>
-      </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t>PDF hat 365 mehr RechNr als BI → PDFs ohne BI-Eintrag</t>
+        <v>4332</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>4078 mehr PDF-Sendungen als BI-Sendungen → PDFs aus anderen Perioden/Kunden</t>
         </is>
       </c>
     </row>
@@ -1000,38 +893,29 @@
         <v>3195</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>73</v>
+        <v>535</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>76</v>
+        <v>543</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>543</v>
+        <v>225</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>225</v>
+        <v>2970</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>93</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>225</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>2970</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>93</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>281</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="N11" s="6" t="inlineStr">
-        <is>
-          <t>BI 43.8 Zeilen/RechNr, PDF 7.1 Pos/RechNr</t>
+        <v>310</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>2660 mehr BI-Sendungen als PDF-Sendungen → fehlende PDFs</t>
         </is>
       </c>
     </row>
@@ -1050,38 +934,29 @@
         <v>641</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>641</v>
+        <v>1779</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1137</v>
+        <v>1854</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1854</v>
+        <v>479</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>479</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>479</v>
+        <v>162</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>25.3</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>479</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="K12" s="5" t="n">
-        <v>25.3</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>1328</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>71.59999999999999</v>
-      </c>
-      <c r="N12" s="6" t="inlineStr">
-        <is>
-          <t>PDF hat 496 mehr RechNr als BI → PDFs ohne BI-Eintrag</t>
+        <v>1300</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>1138 mehr PDF-Sendungen als BI-Sendungen → PDFs aus anderen Perioden/Kunden</t>
         </is>
       </c>
     </row>
@@ -1100,44 +975,35 @@
         <v>790</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>68</v>
+        <v>1191</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>103</v>
+        <v>1191</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>1191</v>
+        <v>555</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>555</v>
+        <v>235</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>29.7</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>555</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>235</v>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="L13" s="4" t="n">
-        <v>508</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>42.7</v>
-      </c>
-      <c r="N13" s="6" t="inlineStr">
-        <is>
-          <t>PDF hat 35 mehr RechNr als BI → PDFs ohne BI-Eintrag</t>
+        <v>636</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>401 mehr PDF-Sendungen als BI-Sendungen → PDFs aus anderen Perioden/Kunden</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>